<commit_message>
eval: Collections AR agent v2 run (80/80, success 6→43) — Radha placeholder fix confirmed, new tool surface observed
- v2 run: accounts/collections/runs/query_results_v2.jsonl, 80/80 OK, avg 16.9s
- Quality: success 43 / marginal 31 / no_data 6 (v1 was 6/70/4) — 7x success gain
- Root cause: live agent shipped NEW tools get_receivables (41 calls) + get_collections (8)
  that are absent from the documented 4-tool allow-list; Overdue & Aging went 0/8 -> 8/8
- Placeholder fix confirmed: Radha Agencies Pvt Ltd 787 now resolves via search_customers_master
  + data tool (was dead-end 'customer not found' with ABC Industries)
- expected_tool mapping is now stale vs real surface (~40 NO_TOOL answered, 8 correct refusals
  marked TOOL); readout recommends regenerating mapping for v3
- EVAL_READOUT_v2.md with full per-category + v1->v2 churn (55%) breakdown
</commit_message>
<xml_diff>
--- a/accounts/collections/queries.xlsx
+++ b/accounts/collections/queries.xlsx
@@ -658,7 +658,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Show me all outstanding invoices for ABC Industries.</t>
+          <t>Show me all outstanding invoices for Radha Agencies Pvt Ltd 787.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -670,7 +670,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>How much does ABC Industries currently owe us?</t>
+          <t>How much does Radha Agencies Pvt Ltd 787 currently owe us?</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>When was the last payment received from ABC Industries?</t>
+          <t>When was the last payment received from Radha Agencies Pvt Ltd 787?</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -694,7 +694,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Show me the payment history of ABC Industries.</t>
+          <t>Show me the payment history of Radha Agencies Pvt Ltd 787.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -706,7 +706,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Does ABC Industries have any invoices overdue by more than 60 days?</t>
+          <t>Does Radha Agencies Pvt Ltd 787 have any invoices overdue by more than 60 days?</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -718,7 +718,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>What is the total invoiced amount versus the amount paid by ABC Industries?</t>
+          <t>What is the total invoiced amount versus the amount paid by Radha Agencies Pvt Ltd 787?</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -730,7 +730,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Has ABC Industries been consistently paying late?</t>
+          <t>Has Radha Agencies Pvt Ltd 787 been consistently paying late?</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -742,7 +742,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Which invoices from ABC Industries are still pending?</t>
+          <t>Which invoices from Radha Agencies Pvt Ltd 787 are still pending?</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">

</xml_diff>